<commit_message>
Refresh import bundles and reports for mainstream-path import
Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-footer.report.xlsx
+++ b/tools/importer/reports/import-footer.report.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="49">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="392" uniqueCount="203">
   <si>
     <t>_reportFile</t>
   </si>
@@ -34,31 +34,340 @@
     <t>url</t>
   </si>
   <si>
+    <t>about-us.report.json</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>about-us</t>
+  </si>
+  <si>
+    <t>success</t>
+  </si>
+  <si>
+    <t>2026-09-09T09:12:39.408Z</t>
+  </si>
+  <si>
+    <t>https://wknd.site/us/en/about-us.html</t>
+  </si>
+  <si>
+    <t>adventures.report.json</t>
+  </si>
+  <si>
+    <t>adventures</t>
+  </si>
+  <si>
+    <t>2026-09-09T09:12:28.181Z</t>
+  </si>
+  <si>
+    <t>https://wknd.site/us/en/adventures.html</t>
+  </si>
+  <si>
+    <t>faqs.report.json</t>
+  </si>
+  <si>
+    <t>faqs</t>
+  </si>
+  <si>
+    <t>2026-09-09T09:12:33.729Z</t>
+  </si>
+  <si>
+    <t>https://wknd.site/us/en/faqs.html</t>
+  </si>
+  <si>
     <t>footer.report.json</t>
   </si>
   <si>
-    <t/>
-  </si>
-  <si>
     <t>footer</t>
   </si>
   <si>
-    <t>success</t>
-  </si>
-  <si>
-    <t>2026-09-09T08:51:40.717Z</t>
+    <t>2026-09-09T09:14:51.878Z</t>
   </si>
   <si>
     <t>https://wknd.site/us/en.html</t>
   </si>
   <si>
+    <t>index.report.json</t>
+  </si>
+  <si>
+    <t>index</t>
+  </si>
+  <si>
+    <t>2026-09-09T09:12:18.599Z</t>
+  </si>
+  <si>
+    <t>magazine.report.json</t>
+  </si>
+  <si>
+    <t>magazine</t>
+  </si>
+  <si>
+    <t>2026-09-09T09:12:22.709Z</t>
+  </si>
+  <si>
+    <t>https://wknd.site/us/en/magazine.html</t>
+  </si>
+  <si>
     <t>nav.report.json</t>
   </si>
   <si>
     <t>nav</t>
   </si>
   <si>
-    <t>2026-09-09T08:51:36.421Z</t>
+    <t>2026-09-09T09:14:46.901Z</t>
+  </si>
+  <si>
+    <t>adventures/bali-surf-camp.report.json</t>
+  </si>
+  <si>
+    <t>adventures/bali-surf-camp</t>
+  </si>
+  <si>
+    <t>2026-09-09T09:13:36.980Z</t>
+  </si>
+  <si>
+    <t>https://wknd.site/us/en/adventures/bali-surf-camp.html</t>
+  </si>
+  <si>
+    <t>adventures/beervana-portland.report.json</t>
+  </si>
+  <si>
+    <t>adventures/beervana-portland</t>
+  </si>
+  <si>
+    <t>2026-09-09T09:13:42.910Z</t>
+  </si>
+  <si>
+    <t>https://wknd.site/us/en/adventures/beervana-portland.html</t>
+  </si>
+  <si>
+    <t>adventures/climbing-new-zealand.report.json</t>
+  </si>
+  <si>
+    <t>adventures/climbing-new-zealand</t>
+  </si>
+  <si>
+    <t>2026-09-09T09:13:13.251Z</t>
+  </si>
+  <si>
+    <t>https://wknd.site/us/en/adventures/climbing-new-zealand.html</t>
+  </si>
+  <si>
+    <t>adventures/colorado-rock-climbing.report.json</t>
+  </si>
+  <si>
+    <t>adventures/colorado-rock-climbing</t>
+  </si>
+  <si>
+    <t>2026-09-09T09:13:47.748Z</t>
+  </si>
+  <si>
+    <t>https://wknd.site/us/en/adventures/colorado-rock-climbing.html</t>
+  </si>
+  <si>
+    <t>adventures/cycling-southern-utah.report.json</t>
+  </si>
+  <si>
+    <t>adventures/cycling-southern-utah</t>
+  </si>
+  <si>
+    <t>2026-09-09T09:13:53.380Z</t>
+  </si>
+  <si>
+    <t>https://wknd.site/us/en/adventures/cycling-southern-utah.html</t>
+  </si>
+  <si>
+    <t>adventures/cycling-tuscany.report.json</t>
+  </si>
+  <si>
+    <t>adventures/cycling-tuscany</t>
+  </si>
+  <si>
+    <t>2026-09-09T09:13:58.848Z</t>
+  </si>
+  <si>
+    <t>https://wknd.site/us/en/adventures/cycling-tuscany.html</t>
+  </si>
+  <si>
+    <t>adventures/downhill-skiing-wyoming.report.json</t>
+  </si>
+  <si>
+    <t>adventures/downhill-skiing-wyoming</t>
+  </si>
+  <si>
+    <t>2026-09-09T09:12:49.473Z</t>
+  </si>
+  <si>
+    <t>https://wknd.site/us/en/adventures/downhill-skiing-wyoming.html</t>
+  </si>
+  <si>
+    <t>adventures/gastronomic-marais-tour.report.json</t>
+  </si>
+  <si>
+    <t>adventures/gastronomic-marais-tour</t>
+  </si>
+  <si>
+    <t>2026-09-09T09:14:04.709Z</t>
+  </si>
+  <si>
+    <t>https://wknd.site/us/en/adventures/gastronomic-marais-tour.html</t>
+  </si>
+  <si>
+    <t>adventures/napa-wine-tasting.report.json</t>
+  </si>
+  <si>
+    <t>adventures/napa-wine-tasting</t>
+  </si>
+  <si>
+    <t>2026-09-09T09:14:09.713Z</t>
+  </si>
+  <si>
+    <t>https://wknd.site/us/en/adventures/napa-wine-tasting.html</t>
+  </si>
+  <si>
+    <t>adventures/riverside-camping-australia.report.json</t>
+  </si>
+  <si>
+    <t>adventures/riverside-camping-australia</t>
+  </si>
+  <si>
+    <t>2026-09-09T09:14:14.158Z</t>
+  </si>
+  <si>
+    <t>https://wknd.site/us/en/adventures/riverside-camping-australia.html</t>
+  </si>
+  <si>
+    <t>adventures/ski-touring-mont-blanc.report.json</t>
+  </si>
+  <si>
+    <t>adventures/ski-touring-mont-blanc</t>
+  </si>
+  <si>
+    <t>2026-09-09T09:14:19.846Z</t>
+  </si>
+  <si>
+    <t>https://wknd.site/us/en/adventures/ski-touring-mont-blanc.html</t>
+  </si>
+  <si>
+    <t>adventures/surf-camp-costa-rica.report.json</t>
+  </si>
+  <si>
+    <t>adventures/surf-camp-costa-rica</t>
+  </si>
+  <si>
+    <t>2026-09-09T09:14:23.721Z</t>
+  </si>
+  <si>
+    <t>https://wknd.site/us/en/adventures/surf-camp-costa-rica.html</t>
+  </si>
+  <si>
+    <t>adventures/tahoe-skiing.report.json</t>
+  </si>
+  <si>
+    <t>adventures/tahoe-skiing</t>
+  </si>
+  <si>
+    <t>2026-09-09T09:13:31.247Z</t>
+  </si>
+  <si>
+    <t>https://wknd.site/us/en/adventures/tahoe-skiing.html</t>
+  </si>
+  <si>
+    <t>adventures/west-coast-cycling.report.json</t>
+  </si>
+  <si>
+    <t>adventures/west-coast-cycling</t>
+  </si>
+  <si>
+    <t>2026-09-09T09:13:26.227Z</t>
+  </si>
+  <si>
+    <t>https://wknd.site/us/en/adventures/west-coast-cycling.html</t>
+  </si>
+  <si>
+    <t>adventures/whistler-mountain-biking.report.json</t>
+  </si>
+  <si>
+    <t>adventures/whistler-mountain-biking</t>
+  </si>
+  <si>
+    <t>2026-09-09T09:13:22.309Z</t>
+  </si>
+  <si>
+    <t>https://wknd.site/us/en/adventures/whistler-mountain-biking.html</t>
+  </si>
+  <si>
+    <t>adventures/yosemite-backpacking.report.json</t>
+  </si>
+  <si>
+    <t>adventures/yosemite-backpacking</t>
+  </si>
+  <si>
+    <t>2026-09-09T09:13:18.259Z</t>
+  </si>
+  <si>
+    <t>https://wknd.site/us/en/adventures/yosemite-backpacking.html</t>
+  </si>
+  <si>
+    <t>magazine/arctic-surfing.report.json</t>
+  </si>
+  <si>
+    <t>magazine/arctic-surfing</t>
+  </si>
+  <si>
+    <t>2026-09-09T09:13:09.344Z</t>
+  </si>
+  <si>
+    <t>https://wknd.site/us/en/magazine/arctic-surfing.html</t>
+  </si>
+  <si>
+    <t>magazine/guide-la-skateparks.report.json</t>
+  </si>
+  <si>
+    <t>magazine/guide-la-skateparks</t>
+  </si>
+  <si>
+    <t>2026-09-09T09:12:59.970Z</t>
+  </si>
+  <si>
+    <t>https://wknd.site/us/en/magazine/guide-la-skateparks.html</t>
+  </si>
+  <si>
+    <t>magazine/san-diego-surf.report.json</t>
+  </si>
+  <si>
+    <t>magazine/san-diego-surf</t>
+  </si>
+  <si>
+    <t>2026-09-09T09:12:44.409Z</t>
+  </si>
+  <si>
+    <t>https://wknd.site/us/en/magazine/san-diego-surf.html</t>
+  </si>
+  <si>
+    <t>magazine/ski-touring.report.json</t>
+  </si>
+  <si>
+    <t>magazine/ski-touring</t>
+  </si>
+  <si>
+    <t>2026-09-09T09:13:05.187Z</t>
+  </si>
+  <si>
+    <t>https://wknd.site/us/en/magazine/ski-touring.html</t>
+  </si>
+  <si>
+    <t>magazine/western-australia.report.json</t>
+  </si>
+  <si>
+    <t>magazine/western-australia</t>
+  </si>
+  <si>
+    <t>2026-09-09T09:12:54.350Z</t>
+  </si>
+  <si>
+    <t>https://wknd.site/us/en/magazine/western-australia.html</t>
   </si>
   <si>
     <t>us/en.html.report.json</t>
@@ -94,9 +403,6 @@
     <t>2026-09-09T08:43:33.336Z</t>
   </si>
   <si>
-    <t>https://wknd.site/us/en/about-us.html</t>
-  </si>
-  <si>
     <t>us/en/adventures.report.json</t>
   </si>
   <si>
@@ -106,9 +412,6 @@
     <t>2026-09-09T08:43:27.395Z</t>
   </si>
   <si>
-    <t>https://wknd.site/us/en/adventures.html</t>
-  </si>
-  <si>
     <t>us/en/faqs.report.json</t>
   </si>
   <si>
@@ -118,9 +421,6 @@
     <t>2026-09-09T08:43:37.609Z</t>
   </si>
   <si>
-    <t>https://wknd.site/us/en/faqs.html</t>
-  </si>
-  <si>
     <t>us/en/index.report.json</t>
   </si>
   <si>
@@ -139,9 +439,6 @@
     <t>2026-09-09T08:48:18.708Z</t>
   </si>
   <si>
-    <t>https://wknd.site/us/en/magazine.html</t>
-  </si>
-  <si>
     <t>us/en/adventures/bali-surf-camp.report.json</t>
   </si>
   <si>
@@ -151,7 +448,139 @@
     <t>2026-09-09T08:43:23.215Z</t>
   </si>
   <si>
-    <t>https://wknd.site/us/en/adventures/bali-surf-camp.html</t>
+    <t>us/en/adventures/beervana-portland.report.json</t>
+  </si>
+  <si>
+    <t>us/en/adventures/beervana-portland</t>
+  </si>
+  <si>
+    <t>2026-09-09T08:54:02.653Z</t>
+  </si>
+  <si>
+    <t>us/en/adventures/climbing-new-zealand.report.json</t>
+  </si>
+  <si>
+    <t>us/en/adventures/climbing-new-zealand</t>
+  </si>
+  <si>
+    <t>2026-09-09T08:53:35.812Z</t>
+  </si>
+  <si>
+    <t>us/en/adventures/colorado-rock-climbing.report.json</t>
+  </si>
+  <si>
+    <t>us/en/adventures/colorado-rock-climbing</t>
+  </si>
+  <si>
+    <t>2026-09-09T08:54:08.350Z</t>
+  </si>
+  <si>
+    <t>us/en/adventures/cycling-southern-utah.report.json</t>
+  </si>
+  <si>
+    <t>us/en/adventures/cycling-southern-utah</t>
+  </si>
+  <si>
+    <t>2026-09-09T08:54:14.066Z</t>
+  </si>
+  <si>
+    <t>us/en/adventures/cycling-tuscany.report.json</t>
+  </si>
+  <si>
+    <t>us/en/adventures/cycling-tuscany</t>
+  </si>
+  <si>
+    <t>2026-09-09T08:54:20.290Z</t>
+  </si>
+  <si>
+    <t>us/en/adventures/downhill-skiing-wyoming.report.json</t>
+  </si>
+  <si>
+    <t>us/en/adventures/downhill-skiing-wyoming</t>
+  </si>
+  <si>
+    <t>2026-09-09T08:53:17.253Z</t>
+  </si>
+  <si>
+    <t>us/en/adventures/gastronomic-marais-tour.report.json</t>
+  </si>
+  <si>
+    <t>us/en/adventures/gastronomic-marais-tour</t>
+  </si>
+  <si>
+    <t>2026-09-09T08:54:25.706Z</t>
+  </si>
+  <si>
+    <t>us/en/adventures/napa-wine-tasting.report.json</t>
+  </si>
+  <si>
+    <t>us/en/adventures/napa-wine-tasting</t>
+  </si>
+  <si>
+    <t>2026-09-09T08:54:32.081Z</t>
+  </si>
+  <si>
+    <t>us/en/adventures/riverside-camping-australia.report.json</t>
+  </si>
+  <si>
+    <t>us/en/adventures/riverside-camping-australia</t>
+  </si>
+  <si>
+    <t>2026-09-09T08:54:37.111Z</t>
+  </si>
+  <si>
+    <t>us/en/adventures/ski-touring-mont-blanc.report.json</t>
+  </si>
+  <si>
+    <t>us/en/adventures/ski-touring-mont-blanc</t>
+  </si>
+  <si>
+    <t>2026-09-09T08:54:41.640Z</t>
+  </si>
+  <si>
+    <t>us/en/adventures/surf-camp-costa-rica.report.json</t>
+  </si>
+  <si>
+    <t>us/en/adventures/surf-camp-costa-rica</t>
+  </si>
+  <si>
+    <t>2026-09-09T08:54:46.066Z</t>
+  </si>
+  <si>
+    <t>us/en/adventures/tahoe-skiing.report.json</t>
+  </si>
+  <si>
+    <t>us/en/adventures/tahoe-skiing</t>
+  </si>
+  <si>
+    <t>2026-09-09T08:53:58.102Z</t>
+  </si>
+  <si>
+    <t>us/en/adventures/west-coast-cycling.report.json</t>
+  </si>
+  <si>
+    <t>us/en/adventures/west-coast-cycling</t>
+  </si>
+  <si>
+    <t>2026-09-09T08:53:52.421Z</t>
+  </si>
+  <si>
+    <t>us/en/adventures/whistler-mountain-biking.report.json</t>
+  </si>
+  <si>
+    <t>us/en/adventures/whistler-mountain-biking</t>
+  </si>
+  <si>
+    <t>2026-09-09T08:53:46.810Z</t>
+  </si>
+  <si>
+    <t>us/en/adventures/yosemite-backpacking.report.json</t>
+  </si>
+  <si>
+    <t>us/en/adventures/yosemite-backpacking</t>
+  </si>
+  <si>
+    <t>2026-09-09T08:53:41.786Z</t>
   </si>
   <si>
     <t>us/en/magazine/arctic-surfing.report.json</t>
@@ -163,7 +592,40 @@
     <t>2026-09-09T08:43:18.057Z</t>
   </si>
   <si>
-    <t>https://wknd.site/us/en/magazine/arctic-surfing.html</t>
+    <t>us/en/magazine/guide-la-skateparks.report.json</t>
+  </si>
+  <si>
+    <t>us/en/magazine/guide-la-skateparks</t>
+  </si>
+  <si>
+    <t>2026-09-09T08:53:26.469Z</t>
+  </si>
+  <si>
+    <t>us/en/magazine/san-diego-surf.report.json</t>
+  </si>
+  <si>
+    <t>us/en/magazine/san-diego-surf</t>
+  </si>
+  <si>
+    <t>2026-09-09T08:53:12.528Z</t>
+  </si>
+  <si>
+    <t>us/en/magazine/ski-touring.report.json</t>
+  </si>
+  <si>
+    <t>us/en/magazine/ski-touring</t>
+  </si>
+  <si>
+    <t>2026-09-09T08:53:30.430Z</t>
+  </si>
+  <si>
+    <t>us/en/magazine/western-australia.report.json</t>
+  </si>
+  <si>
+    <t>us/en/magazine/western-australia</t>
+  </si>
+  <si>
+    <t>2026-09-09T08:53:22.549Z</t>
   </si>
 </sst>
 </file>
@@ -552,12 +1014,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G11"/>
+  <dimension ref="A1:G56"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="1" width="45" customWidth="1"/>
-    <col min="2" max="3" width="50" customWidth="1"/>
-    <col min="4" max="4" width="33" customWidth="1"/>
+    <col min="1" max="3" width="50" customWidth="1"/>
+    <col min="4" max="4" width="46" customWidth="1"/>
     <col min="6" max="6" width="26" customWidth="1"/>
     <col min="7" max="7" width="50" customWidth="1"/>
   </cols>
@@ -628,191 +1089,1226 @@
         <v>15</v>
       </c>
       <c r="G3" t="s">
-        <v>12</v>
+        <v>16</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B4" t="s">
-        <v>17</v>
+        <v>8</v>
       </c>
       <c r="C4" t="s">
+        <v>8</v>
+      </c>
+      <c r="D4" t="s">
         <v>18</v>
       </c>
-      <c r="D4" t="s">
+      <c r="E4" t="s">
+        <v>10</v>
+      </c>
+      <c r="F4" t="s">
         <v>19</v>
       </c>
-      <c r="E4" t="s">
+      <c r="G4" t="s">
         <v>20</v>
-      </c>
-      <c r="F4" t="s">
-        <v>21</v>
-      </c>
-      <c r="G4" t="s">
-        <v>12</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
+        <v>21</v>
+      </c>
+      <c r="B5" t="s">
+        <v>8</v>
+      </c>
+      <c r="C5" t="s">
+        <v>8</v>
+      </c>
+      <c r="D5" t="s">
         <v>22</v>
       </c>
-      <c r="B5" t="s">
-        <v>8</v>
-      </c>
-      <c r="C5" t="s">
-        <v>8</v>
-      </c>
-      <c r="D5" t="s">
+      <c r="E5" t="s">
+        <v>10</v>
+      </c>
+      <c r="F5" t="s">
         <v>23</v>
       </c>
-      <c r="E5" t="s">
-        <v>10</v>
-      </c>
-      <c r="F5" t="s">
+      <c r="G5" t="s">
         <v>24</v>
-      </c>
-      <c r="G5" t="s">
-        <v>25</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
+        <v>25</v>
+      </c>
+      <c r="B6" t="s">
+        <v>8</v>
+      </c>
+      <c r="C6" t="s">
+        <v>8</v>
+      </c>
+      <c r="D6" t="s">
         <v>26</v>
       </c>
-      <c r="B6" t="s">
-        <v>8</v>
-      </c>
-      <c r="C6" t="s">
-        <v>8</v>
-      </c>
-      <c r="D6" t="s">
+      <c r="E6" t="s">
+        <v>10</v>
+      </c>
+      <c r="F6" t="s">
         <v>27</v>
       </c>
-      <c r="E6" t="s">
-        <v>10</v>
-      </c>
-      <c r="F6" t="s">
-        <v>28</v>
-      </c>
       <c r="G6" t="s">
-        <v>29</v>
+        <v>24</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
+        <v>28</v>
+      </c>
+      <c r="B7" t="s">
+        <v>8</v>
+      </c>
+      <c r="C7" t="s">
+        <v>8</v>
+      </c>
+      <c r="D7" t="s">
+        <v>29</v>
+      </c>
+      <c r="E7" t="s">
+        <v>10</v>
+      </c>
+      <c r="F7" t="s">
         <v>30</v>
       </c>
-      <c r="B7" t="s">
-        <v>8</v>
-      </c>
-      <c r="C7" t="s">
-        <v>8</v>
-      </c>
-      <c r="D7" t="s">
+      <c r="G7" t="s">
         <v>31</v>
-      </c>
-      <c r="E7" t="s">
-        <v>10</v>
-      </c>
-      <c r="F7" t="s">
-        <v>32</v>
-      </c>
-      <c r="G7" t="s">
-        <v>33</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
+        <v>32</v>
+      </c>
+      <c r="B8" t="s">
+        <v>8</v>
+      </c>
+      <c r="C8" t="s">
+        <v>8</v>
+      </c>
+      <c r="D8" t="s">
+        <v>33</v>
+      </c>
+      <c r="E8" t="s">
+        <v>10</v>
+      </c>
+      <c r="F8" t="s">
         <v>34</v>
       </c>
-      <c r="B8" t="s">
-        <v>8</v>
-      </c>
-      <c r="C8" t="s">
-        <v>8</v>
-      </c>
-      <c r="D8" t="s">
-        <v>35</v>
-      </c>
-      <c r="E8" t="s">
-        <v>10</v>
-      </c>
-      <c r="F8" t="s">
-        <v>36</v>
-      </c>
       <c r="G8" t="s">
-        <v>12</v>
+        <v>24</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
+        <v>35</v>
+      </c>
+      <c r="B9" t="s">
+        <v>8</v>
+      </c>
+      <c r="C9" t="s">
+        <v>8</v>
+      </c>
+      <c r="D9" t="s">
+        <v>36</v>
+      </c>
+      <c r="E9" t="s">
+        <v>10</v>
+      </c>
+      <c r="F9" t="s">
         <v>37</v>
       </c>
-      <c r="B9" t="s">
-        <v>8</v>
-      </c>
-      <c r="C9" t="s">
-        <v>8</v>
-      </c>
-      <c r="D9" t="s">
+      <c r="G9" t="s">
         <v>38</v>
-      </c>
-      <c r="E9" t="s">
-        <v>10</v>
-      </c>
-      <c r="F9" t="s">
-        <v>39</v>
-      </c>
-      <c r="G9" t="s">
-        <v>40</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
+        <v>39</v>
+      </c>
+      <c r="B10" t="s">
+        <v>8</v>
+      </c>
+      <c r="C10" t="s">
+        <v>8</v>
+      </c>
+      <c r="D10" t="s">
+        <v>40</v>
+      </c>
+      <c r="E10" t="s">
+        <v>10</v>
+      </c>
+      <c r="F10" t="s">
         <v>41</v>
       </c>
-      <c r="B10" t="s">
-        <v>8</v>
-      </c>
-      <c r="C10" t="s">
-        <v>8</v>
-      </c>
-      <c r="D10" t="s">
+      <c r="G10" t="s">
         <v>42</v>
-      </c>
-      <c r="E10" t="s">
-        <v>10</v>
-      </c>
-      <c r="F10" t="s">
-        <v>43</v>
-      </c>
-      <c r="G10" t="s">
-        <v>44</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
+        <v>43</v>
+      </c>
+      <c r="B11" t="s">
+        <v>8</v>
+      </c>
+      <c r="C11" t="s">
+        <v>8</v>
+      </c>
+      <c r="D11" t="s">
+        <v>44</v>
+      </c>
+      <c r="E11" t="s">
+        <v>10</v>
+      </c>
+      <c r="F11" t="s">
         <v>45</v>
       </c>
-      <c r="B11" t="s">
-        <v>8</v>
-      </c>
-      <c r="C11" t="s">
-        <v>8</v>
-      </c>
-      <c r="D11" t="s">
+      <c r="G11" t="s">
         <v>46</v>
       </c>
-      <c r="E11" t="s">
-        <v>10</v>
-      </c>
-      <c r="F11" t="s">
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
         <v>47</v>
       </c>
-      <c r="G11" t="s">
+      <c r="B12" t="s">
+        <v>8</v>
+      </c>
+      <c r="C12" t="s">
+        <v>8</v>
+      </c>
+      <c r="D12" t="s">
         <v>48</v>
+      </c>
+      <c r="E12" t="s">
+        <v>10</v>
+      </c>
+      <c r="F12" t="s">
+        <v>49</v>
+      </c>
+      <c r="G12" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>51</v>
+      </c>
+      <c r="B13" t="s">
+        <v>8</v>
+      </c>
+      <c r="C13" t="s">
+        <v>8</v>
+      </c>
+      <c r="D13" t="s">
+        <v>52</v>
+      </c>
+      <c r="E13" t="s">
+        <v>10</v>
+      </c>
+      <c r="F13" t="s">
+        <v>53</v>
+      </c>
+      <c r="G13" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>55</v>
+      </c>
+      <c r="B14" t="s">
+        <v>8</v>
+      </c>
+      <c r="C14" t="s">
+        <v>8</v>
+      </c>
+      <c r="D14" t="s">
+        <v>56</v>
+      </c>
+      <c r="E14" t="s">
+        <v>10</v>
+      </c>
+      <c r="F14" t="s">
+        <v>57</v>
+      </c>
+      <c r="G14" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>59</v>
+      </c>
+      <c r="B15" t="s">
+        <v>8</v>
+      </c>
+      <c r="C15" t="s">
+        <v>8</v>
+      </c>
+      <c r="D15" t="s">
+        <v>60</v>
+      </c>
+      <c r="E15" t="s">
+        <v>10</v>
+      </c>
+      <c r="F15" t="s">
+        <v>61</v>
+      </c>
+      <c r="G15" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>63</v>
+      </c>
+      <c r="B16" t="s">
+        <v>8</v>
+      </c>
+      <c r="C16" t="s">
+        <v>8</v>
+      </c>
+      <c r="D16" t="s">
+        <v>64</v>
+      </c>
+      <c r="E16" t="s">
+        <v>10</v>
+      </c>
+      <c r="F16" t="s">
+        <v>65</v>
+      </c>
+      <c r="G16" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>67</v>
+      </c>
+      <c r="B17" t="s">
+        <v>8</v>
+      </c>
+      <c r="C17" t="s">
+        <v>8</v>
+      </c>
+      <c r="D17" t="s">
+        <v>68</v>
+      </c>
+      <c r="E17" t="s">
+        <v>10</v>
+      </c>
+      <c r="F17" t="s">
+        <v>69</v>
+      </c>
+      <c r="G17" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>71</v>
+      </c>
+      <c r="B18" t="s">
+        <v>8</v>
+      </c>
+      <c r="C18" t="s">
+        <v>8</v>
+      </c>
+      <c r="D18" t="s">
+        <v>72</v>
+      </c>
+      <c r="E18" t="s">
+        <v>10</v>
+      </c>
+      <c r="F18" t="s">
+        <v>73</v>
+      </c>
+      <c r="G18" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>75</v>
+      </c>
+      <c r="B19" t="s">
+        <v>8</v>
+      </c>
+      <c r="C19" t="s">
+        <v>8</v>
+      </c>
+      <c r="D19" t="s">
+        <v>76</v>
+      </c>
+      <c r="E19" t="s">
+        <v>10</v>
+      </c>
+      <c r="F19" t="s">
+        <v>77</v>
+      </c>
+      <c r="G19" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>79</v>
+      </c>
+      <c r="B20" t="s">
+        <v>8</v>
+      </c>
+      <c r="C20" t="s">
+        <v>8</v>
+      </c>
+      <c r="D20" t="s">
+        <v>80</v>
+      </c>
+      <c r="E20" t="s">
+        <v>10</v>
+      </c>
+      <c r="F20" t="s">
+        <v>81</v>
+      </c>
+      <c r="G20" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>83</v>
+      </c>
+      <c r="B21" t="s">
+        <v>8</v>
+      </c>
+      <c r="C21" t="s">
+        <v>8</v>
+      </c>
+      <c r="D21" t="s">
+        <v>84</v>
+      </c>
+      <c r="E21" t="s">
+        <v>10</v>
+      </c>
+      <c r="F21" t="s">
+        <v>85</v>
+      </c>
+      <c r="G21" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>87</v>
+      </c>
+      <c r="B22" t="s">
+        <v>8</v>
+      </c>
+      <c r="C22" t="s">
+        <v>8</v>
+      </c>
+      <c r="D22" t="s">
+        <v>88</v>
+      </c>
+      <c r="E22" t="s">
+        <v>10</v>
+      </c>
+      <c r="F22" t="s">
+        <v>89</v>
+      </c>
+      <c r="G22" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>91</v>
+      </c>
+      <c r="B23" t="s">
+        <v>8</v>
+      </c>
+      <c r="C23" t="s">
+        <v>8</v>
+      </c>
+      <c r="D23" t="s">
+        <v>92</v>
+      </c>
+      <c r="E23" t="s">
+        <v>10</v>
+      </c>
+      <c r="F23" t="s">
+        <v>93</v>
+      </c>
+      <c r="G23" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>95</v>
+      </c>
+      <c r="B24" t="s">
+        <v>8</v>
+      </c>
+      <c r="C24" t="s">
+        <v>8</v>
+      </c>
+      <c r="D24" t="s">
+        <v>96</v>
+      </c>
+      <c r="E24" t="s">
+        <v>10</v>
+      </c>
+      <c r="F24" t="s">
+        <v>97</v>
+      </c>
+      <c r="G24" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>99</v>
+      </c>
+      <c r="B25" t="s">
+        <v>8</v>
+      </c>
+      <c r="C25" t="s">
+        <v>8</v>
+      </c>
+      <c r="D25" t="s">
+        <v>100</v>
+      </c>
+      <c r="E25" t="s">
+        <v>10</v>
+      </c>
+      <c r="F25" t="s">
+        <v>101</v>
+      </c>
+      <c r="G25" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>103</v>
+      </c>
+      <c r="B26" t="s">
+        <v>8</v>
+      </c>
+      <c r="C26" t="s">
+        <v>8</v>
+      </c>
+      <c r="D26" t="s">
+        <v>104</v>
+      </c>
+      <c r="E26" t="s">
+        <v>10</v>
+      </c>
+      <c r="F26" t="s">
+        <v>105</v>
+      </c>
+      <c r="G26" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>107</v>
+      </c>
+      <c r="B27" t="s">
+        <v>8</v>
+      </c>
+      <c r="C27" t="s">
+        <v>8</v>
+      </c>
+      <c r="D27" t="s">
+        <v>108</v>
+      </c>
+      <c r="E27" t="s">
+        <v>10</v>
+      </c>
+      <c r="F27" t="s">
+        <v>109</v>
+      </c>
+      <c r="G27" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>111</v>
+      </c>
+      <c r="B28" t="s">
+        <v>8</v>
+      </c>
+      <c r="C28" t="s">
+        <v>8</v>
+      </c>
+      <c r="D28" t="s">
+        <v>112</v>
+      </c>
+      <c r="E28" t="s">
+        <v>10</v>
+      </c>
+      <c r="F28" t="s">
+        <v>113</v>
+      </c>
+      <c r="G28" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>115</v>
+      </c>
+      <c r="B29" t="s">
+        <v>8</v>
+      </c>
+      <c r="C29" t="s">
+        <v>8</v>
+      </c>
+      <c r="D29" t="s">
+        <v>116</v>
+      </c>
+      <c r="E29" t="s">
+        <v>10</v>
+      </c>
+      <c r="F29" t="s">
+        <v>117</v>
+      </c>
+      <c r="G29" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>119</v>
+      </c>
+      <c r="B30" t="s">
+        <v>120</v>
+      </c>
+      <c r="C30" t="s">
+        <v>121</v>
+      </c>
+      <c r="D30" t="s">
+        <v>122</v>
+      </c>
+      <c r="E30" t="s">
+        <v>123</v>
+      </c>
+      <c r="F30" t="s">
+        <v>124</v>
+      </c>
+      <c r="G30" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>125</v>
+      </c>
+      <c r="B31" t="s">
+        <v>8</v>
+      </c>
+      <c r="C31" t="s">
+        <v>8</v>
+      </c>
+      <c r="D31" t="s">
+        <v>126</v>
+      </c>
+      <c r="E31" t="s">
+        <v>10</v>
+      </c>
+      <c r="F31" t="s">
+        <v>127</v>
+      </c>
+      <c r="G31" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>128</v>
+      </c>
+      <c r="B32" t="s">
+        <v>8</v>
+      </c>
+      <c r="C32" t="s">
+        <v>8</v>
+      </c>
+      <c r="D32" t="s">
+        <v>129</v>
+      </c>
+      <c r="E32" t="s">
+        <v>10</v>
+      </c>
+      <c r="F32" t="s">
+        <v>130</v>
+      </c>
+      <c r="G32" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="33" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>131</v>
+      </c>
+      <c r="B33" t="s">
+        <v>8</v>
+      </c>
+      <c r="C33" t="s">
+        <v>8</v>
+      </c>
+      <c r="D33" t="s">
+        <v>132</v>
+      </c>
+      <c r="E33" t="s">
+        <v>10</v>
+      </c>
+      <c r="F33" t="s">
+        <v>133</v>
+      </c>
+      <c r="G33" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="34" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>134</v>
+      </c>
+      <c r="B34" t="s">
+        <v>8</v>
+      </c>
+      <c r="C34" t="s">
+        <v>8</v>
+      </c>
+      <c r="D34" t="s">
+        <v>135</v>
+      </c>
+      <c r="E34" t="s">
+        <v>10</v>
+      </c>
+      <c r="F34" t="s">
+        <v>136</v>
+      </c>
+      <c r="G34" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>137</v>
+      </c>
+      <c r="B35" t="s">
+        <v>8</v>
+      </c>
+      <c r="C35" t="s">
+        <v>8</v>
+      </c>
+      <c r="D35" t="s">
+        <v>138</v>
+      </c>
+      <c r="E35" t="s">
+        <v>10</v>
+      </c>
+      <c r="F35" t="s">
+        <v>139</v>
+      </c>
+      <c r="G35" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="36" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>140</v>
+      </c>
+      <c r="B36" t="s">
+        <v>8</v>
+      </c>
+      <c r="C36" t="s">
+        <v>8</v>
+      </c>
+      <c r="D36" t="s">
+        <v>141</v>
+      </c>
+      <c r="E36" t="s">
+        <v>10</v>
+      </c>
+      <c r="F36" t="s">
+        <v>142</v>
+      </c>
+      <c r="G36" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="37" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
+        <v>143</v>
+      </c>
+      <c r="B37" t="s">
+        <v>8</v>
+      </c>
+      <c r="C37" t="s">
+        <v>8</v>
+      </c>
+      <c r="D37" t="s">
+        <v>144</v>
+      </c>
+      <c r="E37" t="s">
+        <v>10</v>
+      </c>
+      <c r="F37" t="s">
+        <v>145</v>
+      </c>
+      <c r="G37" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="38" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
+        <v>146</v>
+      </c>
+      <c r="B38" t="s">
+        <v>8</v>
+      </c>
+      <c r="C38" t="s">
+        <v>8</v>
+      </c>
+      <c r="D38" t="s">
+        <v>147</v>
+      </c>
+      <c r="E38" t="s">
+        <v>10</v>
+      </c>
+      <c r="F38" t="s">
+        <v>148</v>
+      </c>
+      <c r="G38" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="39" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
+        <v>149</v>
+      </c>
+      <c r="B39" t="s">
+        <v>8</v>
+      </c>
+      <c r="C39" t="s">
+        <v>8</v>
+      </c>
+      <c r="D39" t="s">
+        <v>150</v>
+      </c>
+      <c r="E39" t="s">
+        <v>10</v>
+      </c>
+      <c r="F39" t="s">
+        <v>151</v>
+      </c>
+      <c r="G39" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="40" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A40" t="s">
+        <v>152</v>
+      </c>
+      <c r="B40" t="s">
+        <v>8</v>
+      </c>
+      <c r="C40" t="s">
+        <v>8</v>
+      </c>
+      <c r="D40" t="s">
+        <v>153</v>
+      </c>
+      <c r="E40" t="s">
+        <v>10</v>
+      </c>
+      <c r="F40" t="s">
+        <v>154</v>
+      </c>
+      <c r="G40" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="41" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
+        <v>155</v>
+      </c>
+      <c r="B41" t="s">
+        <v>8</v>
+      </c>
+      <c r="C41" t="s">
+        <v>8</v>
+      </c>
+      <c r="D41" t="s">
+        <v>156</v>
+      </c>
+      <c r="E41" t="s">
+        <v>10</v>
+      </c>
+      <c r="F41" t="s">
+        <v>157</v>
+      </c>
+      <c r="G41" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="42" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
+        <v>158</v>
+      </c>
+      <c r="B42" t="s">
+        <v>8</v>
+      </c>
+      <c r="C42" t="s">
+        <v>8</v>
+      </c>
+      <c r="D42" t="s">
+        <v>159</v>
+      </c>
+      <c r="E42" t="s">
+        <v>10</v>
+      </c>
+      <c r="F42" t="s">
+        <v>160</v>
+      </c>
+      <c r="G42" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="43" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A43" t="s">
+        <v>161</v>
+      </c>
+      <c r="B43" t="s">
+        <v>8</v>
+      </c>
+      <c r="C43" t="s">
+        <v>8</v>
+      </c>
+      <c r="D43" t="s">
+        <v>162</v>
+      </c>
+      <c r="E43" t="s">
+        <v>10</v>
+      </c>
+      <c r="F43" t="s">
+        <v>163</v>
+      </c>
+      <c r="G43" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="44" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A44" t="s">
+        <v>164</v>
+      </c>
+      <c r="B44" t="s">
+        <v>8</v>
+      </c>
+      <c r="C44" t="s">
+        <v>8</v>
+      </c>
+      <c r="D44" t="s">
+        <v>165</v>
+      </c>
+      <c r="E44" t="s">
+        <v>10</v>
+      </c>
+      <c r="F44" t="s">
+        <v>166</v>
+      </c>
+      <c r="G44" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="45" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A45" t="s">
+        <v>167</v>
+      </c>
+      <c r="B45" t="s">
+        <v>8</v>
+      </c>
+      <c r="C45" t="s">
+        <v>8</v>
+      </c>
+      <c r="D45" t="s">
+        <v>168</v>
+      </c>
+      <c r="E45" t="s">
+        <v>10</v>
+      </c>
+      <c r="F45" t="s">
+        <v>169</v>
+      </c>
+      <c r="G45" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="46" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A46" t="s">
+        <v>170</v>
+      </c>
+      <c r="B46" t="s">
+        <v>8</v>
+      </c>
+      <c r="C46" t="s">
+        <v>8</v>
+      </c>
+      <c r="D46" t="s">
+        <v>171</v>
+      </c>
+      <c r="E46" t="s">
+        <v>10</v>
+      </c>
+      <c r="F46" t="s">
+        <v>172</v>
+      </c>
+      <c r="G46" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="47" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A47" t="s">
+        <v>173</v>
+      </c>
+      <c r="B47" t="s">
+        <v>8</v>
+      </c>
+      <c r="C47" t="s">
+        <v>8</v>
+      </c>
+      <c r="D47" t="s">
+        <v>174</v>
+      </c>
+      <c r="E47" t="s">
+        <v>10</v>
+      </c>
+      <c r="F47" t="s">
+        <v>175</v>
+      </c>
+      <c r="G47" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="48" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A48" t="s">
+        <v>176</v>
+      </c>
+      <c r="B48" t="s">
+        <v>8</v>
+      </c>
+      <c r="C48" t="s">
+        <v>8</v>
+      </c>
+      <c r="D48" t="s">
+        <v>177</v>
+      </c>
+      <c r="E48" t="s">
+        <v>10</v>
+      </c>
+      <c r="F48" t="s">
+        <v>178</v>
+      </c>
+      <c r="G48" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="49" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A49" t="s">
+        <v>179</v>
+      </c>
+      <c r="B49" t="s">
+        <v>8</v>
+      </c>
+      <c r="C49" t="s">
+        <v>8</v>
+      </c>
+      <c r="D49" t="s">
+        <v>180</v>
+      </c>
+      <c r="E49" t="s">
+        <v>10</v>
+      </c>
+      <c r="F49" t="s">
+        <v>181</v>
+      </c>
+      <c r="G49" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="50" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A50" t="s">
+        <v>182</v>
+      </c>
+      <c r="B50" t="s">
+        <v>8</v>
+      </c>
+      <c r="C50" t="s">
+        <v>8</v>
+      </c>
+      <c r="D50" t="s">
+        <v>183</v>
+      </c>
+      <c r="E50" t="s">
+        <v>10</v>
+      </c>
+      <c r="F50" t="s">
+        <v>184</v>
+      </c>
+      <c r="G50" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="51" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A51" t="s">
+        <v>185</v>
+      </c>
+      <c r="B51" t="s">
+        <v>8</v>
+      </c>
+      <c r="C51" t="s">
+        <v>8</v>
+      </c>
+      <c r="D51" t="s">
+        <v>186</v>
+      </c>
+      <c r="E51" t="s">
+        <v>10</v>
+      </c>
+      <c r="F51" t="s">
+        <v>187</v>
+      </c>
+      <c r="G51" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="52" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A52" t="s">
+        <v>188</v>
+      </c>
+      <c r="B52" t="s">
+        <v>8</v>
+      </c>
+      <c r="C52" t="s">
+        <v>8</v>
+      </c>
+      <c r="D52" t="s">
+        <v>189</v>
+      </c>
+      <c r="E52" t="s">
+        <v>10</v>
+      </c>
+      <c r="F52" t="s">
+        <v>190</v>
+      </c>
+      <c r="G52" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="53" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A53" t="s">
+        <v>191</v>
+      </c>
+      <c r="B53" t="s">
+        <v>8</v>
+      </c>
+      <c r="C53" t="s">
+        <v>8</v>
+      </c>
+      <c r="D53" t="s">
+        <v>192</v>
+      </c>
+      <c r="E53" t="s">
+        <v>10</v>
+      </c>
+      <c r="F53" t="s">
+        <v>193</v>
+      </c>
+      <c r="G53" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="54" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A54" t="s">
+        <v>194</v>
+      </c>
+      <c r="B54" t="s">
+        <v>8</v>
+      </c>
+      <c r="C54" t="s">
+        <v>8</v>
+      </c>
+      <c r="D54" t="s">
+        <v>195</v>
+      </c>
+      <c r="E54" t="s">
+        <v>10</v>
+      </c>
+      <c r="F54" t="s">
+        <v>196</v>
+      </c>
+      <c r="G54" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="55" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A55" t="s">
+        <v>197</v>
+      </c>
+      <c r="B55" t="s">
+        <v>8</v>
+      </c>
+      <c r="C55" t="s">
+        <v>8</v>
+      </c>
+      <c r="D55" t="s">
+        <v>198</v>
+      </c>
+      <c r="E55" t="s">
+        <v>10</v>
+      </c>
+      <c r="F55" t="s">
+        <v>199</v>
+      </c>
+      <c r="G55" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="56" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A56" t="s">
+        <v>200</v>
+      </c>
+      <c r="B56" t="s">
+        <v>8</v>
+      </c>
+      <c r="C56" t="s">
+        <v>8</v>
+      </c>
+      <c r="D56" t="s">
+        <v>201</v>
+      </c>
+      <c r="E56" t="s">
+        <v>10</v>
+      </c>
+      <c r="F56" t="s">
+        <v>202</v>
+      </c>
+      <c r="G56" t="s">
+        <v>118</v>
       </c>
     </row>
   </sheetData>

</xml_diff>